<commit_message>
feat: add text input processing for financial data extraction in FinanceMapper component
</commit_message>
<xml_diff>
--- a/llm_agent_mcp-main/data/sar_8.xlsx
+++ b/llm_agent_mcp-main/data/sar_8.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -580,6 +580,96 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Номин супермаркетаас</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Зарлага</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Хэрэгсэл</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Өнөөдөр Номин супермаркетаас оффисын хэрэгсэлд 45,000 төгрөг зарцуулсан</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Баянбүрд ХХК</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Зарлага</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Түрээс</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Баянбүрд ХХК-аас декабрийн түрээсийн төлбөр 2,500,000 төгрөгийг шилжүүлсэн</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Энэ</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>450000</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Орлого</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Урамшуулал</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Энэ сард цалингаас гадна 300,000 төгрөгийн урамшуулал авсан. Мөн 150,000 төгрөгөөр хоол хүнс авсан.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: streamline finance and conversation routes in api-server
</commit_message>
<xml_diff>
--- a/llm_agent_mcp-main/data/sar_8.xlsx
+++ b/llm_agent_mcp-main/data/sar_8.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -670,6 +670,36 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Тэмүүлэн ХХК</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Зарлага</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Оффис</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Тэмүүлэн ХХК-д интернетийн төлбөр 120,000 төгрөг төлсөн</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add python-docx package metadata and license files
- Created REQUESTED file for python-docx version 1.2.0
- Added WHEEL file for python-docx package distribution
- Included LICENSE file with MIT License details for python-docx
- Added top_level.txt to specify the main module of the package
</commit_message>
<xml_diff>
--- a/llm_agent_mcp-main/data/sar_8.xlsx
+++ b/llm_agent_mcp-main/data/sar_8.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,6 +700,36 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Номин супермаркетаас</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Зарлага</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Хэрэгсэл</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Өнөөдөр Номин супермаркетаас оффисын хэрэгсэлд 45,000 төгрөг зарцуулсан</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update API routes for whatif and history, and allow text/plain uploads
</commit_message>
<xml_diff>
--- a/llm_agent_mcp-main/data/sar_8.xlsx
+++ b/llm_agent_mcp-main/data/sar_8.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -730,6 +730,62 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Номин супермаркетаас</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Зарлага</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Хэрэгсэл</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Өнөөдөр Номин супермаркетаас оффисын хэрэгсэлд 45,000 төгрөг зарцуулсан</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Зарлага</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Бусад</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>test content</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>